<commit_message>
update to sp documents
</commit_message>
<xml_diff>
--- a/exports/NPFR_Strategic_Plan_2026-Q2.xlsx
+++ b/exports/NPFR_Strategic_Plan_2026-Q2.xlsx
@@ -952,7 +952,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Operational Readiness and Deployment  —  Steward: Scott Lane  (2/46 tasks, 4%)</t>
+          <t>Operational Readiness and Deployment  —  Steward: Scott Lane  (4/46 tasks, 9%)</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Workforce Development and Succession  —  Steward: Nick Herlihy  (7/71 tasks, 10%)</t>
+          <t>Workforce Development and Succession  —  Steward: Nick Herlihy  (11/71 tasks, 15%)</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Community Risk Reduction and Public Education  —  Steward: Nick Satterly  (0/44 tasks, 0%)</t>
+          <t>Community Risk Reduction and Public Education  —  Steward: Nick Satterly  (5/44 tasks, 11%)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Professional Standards and Service Excellence  —  Steward: Rick Wilbert  (9/55 tasks, 16%)</t>
+          <t>Professional Standards and Service Excellence  —  Steward: Rick Wilbert  (12/55 tasks, 22%)</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       <c r="A29" s="1" t="n"/>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Generated June 12, 2026  ·  Restructured â€” 4 pillars, 12 domains</t>
+          <t>Generated June 14, 2026  ·  Restructured â€” 4 pillars, 12 domains</t>
         </is>
       </c>
     </row>
@@ -1233,10 +1233,10 @@
         <v>46</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H4" s="16" t="n">
-        <v>0.04347826086956522</v>
+        <v>0.08695652173913043</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -1262,10 +1262,10 @@
         <v>71</v>
       </c>
       <c r="G5" s="18" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>0.09859154929577464</v>
+        <v>0.1549295774647887</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -1291,10 +1291,10 @@
         <v>44</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>0</v>
+        <v>0.1136363636363636</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -1320,10 +1320,10 @@
         <v>55</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H7" s="19" t="n">
-        <v>0.1636363636363636</v>
+        <v>0.2181818181818182</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -1336,10 +1336,10 @@
         <v>216</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.1481481481481481</v>
       </c>
     </row>
   </sheetData>
@@ -1450,7 +1450,11 @@
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G5" s="28" t="inlineStr"/>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>Major incident response plans validated through at least one full-scale or functional drill by Q4, with after-action documentation on file.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="B6" s="13" t="inlineStr">
@@ -1478,7 +1482,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G6" s="33" t="inlineStr"/>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>Station facility maintenance monitoring program operational by Q4, with all items inventoried by responsible party, service schedules documented, and internal tracking system active.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="13" t="inlineStr">
@@ -1506,7 +1514,11 @@
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G7" s="28" t="inlineStr"/>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>Written department-wide succession plan adopted by Q4, identifying all personnel eligible to separate within five years, mapping critical position vacancies, and assigning developmental actions to identified successors.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="B8" s="13" t="inlineStr">
@@ -1534,7 +1546,11 @@
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G8" s="33" t="inlineStr"/>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>Revised Officer Development Program relaunched by Q4 with updated curriculum, current competency expectations aligned to CFAI credentialing categories, and a documented delivery schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="B9" s="13" t="inlineStr">
@@ -1557,12 +1573,16 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F9" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="inlineStr"/>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="inlineStr">
+        <is>
+          <t>Documented roles, responsibilities, and reporting structure established for all training division positions, and continuous evaluation framework for workload and span of control implemented by Q3.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="B10" s="13" t="inlineStr">
@@ -1590,7 +1610,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="G10" s="33" t="inlineStr"/>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>Recruitment program operational by Q4 with formal partnerships at a minimum of four local technical schools, functioning online portal, standardized interview questions, documented scoring system, and active recruitment committee.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="B11" s="13" t="inlineStr">
@@ -1613,12 +1637,16 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F11" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="inlineStr"/>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr">
+        <is>
+          <t>Ranked baseline risk report identifying highest-priority program areas delivered to the CRR team by Q2, drawing from a minimum of five data sources.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="B12" s="13" t="inlineStr">
@@ -1641,12 +1669,16 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F12" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G12" s="33" t="inlineStr"/>
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>Elementary School CRR Education program and Senior Public Education program both operational by Q4, with baseline data collection underway for each.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="B13" s="13" t="inlineStr">
@@ -1669,12 +1701,16 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F13" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="inlineStr"/>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="inlineStr">
+        <is>
+          <t>CFAI candidate application submitted by Q4, with Accreditation SOG formalized and documented proof of compliance gathered across all applicable categories.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="13" t="inlineStr">
@@ -1702,7 +1738,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="G14" s="33" t="inlineStr"/>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>ISO 1 annual compliance package complete by Q4, with all required data documented and site visit readiness package delivered.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="B15" s="13" t="inlineStr">
@@ -1730,7 +1770,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="G15" s="28" t="inlineStr"/>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>Mission Lifeline Gold Rating application submitted by Q4 with supporting quarterly cardiac care data and protocol alignment verified.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="22" t="inlineStr">
@@ -1789,7 +1833,7 @@
       </c>
       <c r="E19" s="26" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Terry McCloud</t>
         </is>
       </c>
       <c r="F19" s="32" t="inlineStr">
@@ -1797,7 +1841,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G19" s="28" t="inlineStr"/>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>Minimum three additional Hazardous Materials Technician-certified personnel achieved, target hazard pre-plan library complete for all identified city sites, and at least one HOT training or tabletop exercise conducted by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="B20" s="13" t="inlineStr">
@@ -1825,7 +1873,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G20" s="33" t="inlineStr"/>
+      <c r="G20" s="33" t="inlineStr">
+        <is>
+          <t>PPE inventory assessed, minimum reserve standards established, lifecycle replacement model documented with annual funding projections, and sustainable PPE readiness program implemented by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="B21" s="13" t="inlineStr">
@@ -1853,7 +1905,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G21" s="28" t="inlineStr"/>
+      <c r="G21" s="28" t="inlineStr">
+        <is>
+          <t>Needs assessment complete, logistics resource hub program developed with inventory management system installed, SOGs documented, personnel trained, and initial effectiveness evaluation completed by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="B22" s="13" t="inlineStr">
@@ -1881,7 +1937,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G22" s="33" t="inlineStr"/>
+      <c r="G22" s="33" t="inlineStr">
+        <is>
+          <t>Comprehensive EMS organizational evaluation complete by Q3, with findings and specific staffing recommendations for QA/QI, accreditation, and specialty program positions presented to command staff.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="B23" s="13" t="inlineStr">
@@ -1909,7 +1969,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G23" s="28" t="inlineStr"/>
+      <c r="G23" s="28" t="inlineStr">
+        <is>
+          <t>Feasibility report on NPFR-hosted training academy presented to command staff by Q4, with recommended implementation pathway, cost estimates, and regional partnership options documented.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="B24" s="13" t="inlineStr">
@@ -1937,7 +2001,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G24" s="33" t="inlineStr"/>
+      <c r="G24" s="33" t="inlineStr">
+        <is>
+          <t>Sleep health evaluation complete by Q4, with findings on crew-quarters configuration, personnel survey results, and facility and policy recommendations presented to command staff.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="B25" s="13" t="inlineStr">
@@ -1965,7 +2033,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G25" s="28" t="inlineStr"/>
+      <c r="G25" s="28" t="inlineStr">
+        <is>
+          <t>Internal communication program fully operational by Q4, with all stations visited a minimum of twice, quarterly department periodical published, and digital communication platform active for shift-based staff.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="B26" s="13" t="inlineStr">
@@ -1993,7 +2065,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G26" s="33" t="inlineStr"/>
+      <c r="G26" s="33" t="inlineStr">
+        <is>
+          <t>Targeted EMS prevention initiatives addressing CPR, falls, stroke awareness, drowning prevention, and severe weather preparedness launched by Q3, with performance measures established for all EMS-related CRR activities.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="B27" s="13" t="inlineStr">
@@ -2021,7 +2097,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G27" s="28" t="inlineStr"/>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>Minimum three new CRR program policies with supporting content complete by Q1, Programs 1 and 2 operational by Q3, and Programs 3 and 4 operational by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="B28" s="13" t="inlineStr">
@@ -2049,7 +2129,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G28" s="33" t="inlineStr"/>
+      <c r="G28" s="33" t="inlineStr">
+        <is>
+          <t>CRR staffing capacity analysis presented to command staff by Q3, and interim capacity solutions including cross-training and volunteer engagement established by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="B29" s="13" t="inlineStr">
@@ -2077,7 +2161,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G29" s="28" t="inlineStr"/>
+      <c r="G29" s="28" t="inlineStr">
+        <is>
+          <t>All assigned accreditation tasks completed, 11th edition manual requirements incorporated, and next defined CFAI accreditation milestone reached by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="B30" s="13" t="inlineStr">
@@ -2092,7 +2180,7 @@
       </c>
       <c r="D30" s="30" t="inlineStr">
         <is>
-          <t>Complete CAAS re-accreditation by incorporating all 4th edition manual requirements, obtaining annual proofs of compliance across all applicable categories, submitting the re-accreditation application, completing the PedReady renewal, and achieving a successful on-site review by Q4.</t>
+          <t>Complete CAAS re-accreditation by incorporating all 4th edition manual requirements, obtaining annual proofs of compliance across all applicable categories, submitting the re-accreditation application, and achieving a successful on-site review by Q4.</t>
         </is>
       </c>
       <c r="E30" s="31" t="inlineStr">
@@ -2105,7 +2193,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G30" s="33" t="inlineStr"/>
+      <c r="G30" s="33" t="inlineStr">
+        <is>
+          <t>CAAS re-accreditation achieved by Q4, with 4th edition manual requirements incorporated, all annual proofs of compliance gathered, re-accreditation application submitted, and successful on-site review conducted.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="B31" s="13" t="inlineStr">
@@ -2133,7 +2225,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G31" s="28" t="inlineStr"/>
+      <c r="G31" s="28" t="inlineStr">
+        <is>
+          <t>ALS coverage improvement plan with specific resource and staffing recommendations presented to executive leadership by Q4, based on completed response time analysis, coverage gap mapping, and staffing model evaluation.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="22" t="inlineStr">
@@ -2202,7 +2298,7 @@
       </c>
       <c r="G35" s="28" t="inlineStr">
         <is>
-          <t>Continuity plan adopted with guides for all critical functions. Depends on completion of both PPE program (P1.27.G2) and logistics hubs program (P1.27.G3).</t>
+          <t>Logistics Division continuity plan adopted with position-specific guides and SOPs for all critical functions, cross-training program established, and program appraisal completed by Q4.</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2328,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G36" s="33" t="inlineStr"/>
+      <c r="G36" s="33" t="inlineStr">
+        <is>
+          <t>Structured assessment of all mutual aid agreements, radio interoperability, and CAD integration complete, with prioritized gap report delivered to command staff by Q2.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="B37" s="13" t="inlineStr">
@@ -2260,7 +2360,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G37" s="28" t="inlineStr"/>
+      <c r="G37" s="28" t="inlineStr">
+        <is>
+          <t>Updated mutual aid agreements, joint training protocols, and communications interoperability solutions developed and delivered to all partner agencies for review by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="B38" s="13" t="inlineStr">
@@ -2288,7 +2392,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G38" s="33" t="inlineStr"/>
+      <c r="G38" s="33" t="inlineStr">
+        <is>
+          <t>EMS supervisory evaluation complete by Q4, with findings on field coverage effectiveness, clinical oversight opportunities, and implementation recommendations for future supervisory positions presented to command staff.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="B39" s="13" t="inlineStr">
@@ -2316,7 +2424,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G39" s="28" t="inlineStr"/>
+      <c r="G39" s="28" t="inlineStr">
+        <is>
+          <t>Formal partnership agreements executed with a minimum of four regional educational institutions by Q4, shared-resource access protocols documented, and joint recruitment pipeline established with at least two institutions.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="B40" s="13" t="inlineStr">
@@ -2344,7 +2456,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G40" s="33" t="inlineStr"/>
+      <c r="G40" s="33" t="inlineStr">
+        <is>
+          <t>NPFR Training Academy established by Q4, with facility and partnership agreements in place and a minimum of one formally structured training program delivered to internal personnel with outcomes documented.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="B41" s="13" t="inlineStr">
@@ -2372,7 +2488,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G41" s="28" t="inlineStr"/>
+      <c r="G41" s="28" t="inlineStr">
+        <is>
+          <t>Individual sleeping room retrofit at Brix station complete by Q4, station-level sleep hygiene protocols adopted, and personnel survey conducted to assess improvement in self-reported sleep quality.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="B42" s="13" t="inlineStr">
@@ -2400,7 +2520,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G42" s="33" t="inlineStr"/>
+      <c r="G42" s="33" t="inlineStr">
+        <is>
+          <t>Written report documenting CRR and EMS program strengths, weaknesses, and data-driven improvement recommendations delivered by Q4, based on updated multi-source data analysis.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="B43" s="13" t="inlineStr">
@@ -2428,7 +2552,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G43" s="28" t="inlineStr"/>
+      <c r="G43" s="28" t="inlineStr">
+        <is>
+          <t>Fire Explorer and Cadet pathway program established in partnership with a minimum of two local high schools by Q4, annual station visits and career days implemented, and formal program appraisal of Cadet Program completed.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="B44" s="13" t="inlineStr">
@@ -2456,7 +2584,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G44" s="33" t="inlineStr"/>
+      <c r="G44" s="33" t="inlineStr">
+        <is>
+          <t>Community Outreach Team established with defined structure and trained membership by Q4, and a minimum of two community events delivered.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="28" customHeight="1">
       <c r="B45" s="13" t="inlineStr">
@@ -2484,7 +2616,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G45" s="28" t="inlineStr"/>
+      <c r="G45" s="28" t="inlineStr">
+        <is>
+          <t>Centralized digital records management system operational by Q4, with complete record inventory documented, all active records migrated, and records meeting retention requirements dispositioned with the Clerk's office.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="28" customHeight="1">
       <c r="B46" s="13" t="inlineStr">
@@ -2512,7 +2648,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G46" s="33" t="inlineStr"/>
+      <c r="G46" s="33" t="inlineStr">
+        <is>
+          <t>MIH implementation recommendation presented to command staff by Q4, with completed operational framework, target population analysis, partner identification, performance measures, referral pathways, and financial and staffing feasibility evaluation.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="28" customHeight="1">
       <c r="B47" s="13" t="inlineStr">
@@ -2540,7 +2680,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G47" s="28" t="inlineStr"/>
+      <c r="G47" s="28" t="inlineStr">
+        <is>
+          <t>Prioritized implementation strategy with go/no-go recommendations for a minimum of two advanced EMS service models presented to executive leadership by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="B49" s="22" t="inlineStr">
@@ -2607,7 +2751,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G51" s="28" t="inlineStr"/>
+      <c r="G51" s="28" t="inlineStr">
+        <is>
+          <t>Fleet readiness and maintenance assessment complete by Q4, with annual maintenance costs calculated per apparatus, downtime measured against manufacturer PM schedules, highest-burden units identified, and KPIs for apparatus availability established.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="28" customHeight="1">
       <c r="B52" s="13" t="inlineStr">
@@ -2635,7 +2783,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G52" s="33" t="inlineStr"/>
+      <c r="G52" s="33" t="inlineStr">
+        <is>
+          <t>Signed updates to all mutual aid agreements executed, minimum one joint interagency training exercise delivered, and communications interoperability verified with all primary mutual aid partners by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="28" customHeight="1">
       <c r="B53" s="13" t="inlineStr">
@@ -2663,7 +2815,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G53" s="28" t="inlineStr"/>
+      <c r="G53" s="28" t="inlineStr">
+        <is>
+          <t>90% or greater professional credentialing of all applicable positions documented by Q4, with individual completion plans on file for all remaining uncredentialed personnel.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="B54" s="13" t="inlineStr">
@@ -2691,7 +2847,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G54" s="33" t="inlineStr"/>
+      <c r="G54" s="33" t="inlineStr">
+        <is>
+          <t>Workforce growth plan presented to command staff by Q4, projecting staffing needs through FY32 with a phased onboarding model covering hiring timeline, employment terms, career progression, and retention strategies.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="28" customHeight="1">
       <c r="B55" s="13" t="inlineStr">
@@ -2719,7 +2879,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G55" s="28" t="inlineStr"/>
+      <c r="G55" s="28" t="inlineStr">
+        <is>
+          <t>Financial plan addressing projected staffing growth through FY32 presented for command staff adoption by Q4, with position cost modeling, identified funding sources, and phased hiring timeline aligned to call volume thresholds.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="28" customHeight="1">
       <c r="B56" s="13" t="inlineStr">
@@ -2747,7 +2911,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G56" s="33" t="inlineStr"/>
+      <c r="G56" s="33" t="inlineStr">
+        <is>
+          <t>Recognized training center status achieved, minimum two training sessions hosted, collaborative training events with external agencies increased 50% over FY28 baseline, and external trainee participation in NPFR-led courses increased 30% by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="B57" s="13" t="inlineStr">
@@ -2775,7 +2943,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G57" s="28" t="inlineStr"/>
+      <c r="G57" s="28" t="inlineStr">
+        <is>
+          <t>Expansion of the three highest-performing CRR programs documented and reported by Q2, with measurable increases in reach, delivery frequency, or target population coverage.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="B58" s="13" t="inlineStr">
@@ -2803,7 +2975,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G58" s="33" t="inlineStr"/>
+      <c r="G58" s="33" t="inlineStr">
+        <is>
+          <t>Improvement plans for the three lowest-performing CRR programs implemented and outcomes assessed by Q3.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="28" customHeight="1">
       <c r="B59" s="13" t="inlineStr">
@@ -2831,7 +3007,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G59" s="28" t="inlineStr"/>
+      <c r="G59" s="28" t="inlineStr">
+        <is>
+          <t>Adapted or new program delivery operational in a minimum of two identified underserved geographic areas or demographic gap populations by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="B60" s="13" t="inlineStr">
@@ -2859,7 +3039,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G60" s="33" t="inlineStr"/>
+      <c r="G60" s="33" t="inlineStr">
+        <is>
+          <t>Historical and Archive Committee established with formal mandate, recruited membership, and initial inventory of historical items complete by Q2; agency performance standards implemented with documented compliance tracking process by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="28" customHeight="1">
       <c r="B61" s="13" t="inlineStr">
@@ -2887,7 +3071,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G61" s="28" t="inlineStr"/>
+      <c r="G61" s="28" t="inlineStr">
+        <is>
+          <t>MIH pilot program launched by Q4 serving identified high-utilizer or at-risk populations, with formal healthcare partnerships established, policy and documentation frameworks complete, and quarterly outcomes tracking initiated.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="28" customHeight="1">
       <c r="B62" s="13" t="inlineStr">
@@ -2915,7 +3103,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G62" s="33" t="inlineStr"/>
+      <c r="G62" s="33" t="inlineStr">
+        <is>
+          <t>Minimum one advanced EMS service model implemented by Q4, with documented operational framework, trained personnel, structured outcomes tracking, and first-year performance report delivered to command staff.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3083,7 +3275,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="K6" s="42" t="inlineStr"/>
+      <c r="K6" s="42" t="inlineStr">
+        <is>
+          <t>Major incident response plans validated through at least one full-scale or functional drill by Q4, with after-action documentation on file.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="H7" s="41" t="inlineStr">
@@ -3113,9 +3309,9 @@
           <t>Plan and conduct a large-scale drill including active shooter scenario.</t>
         </is>
       </c>
-      <c r="J8" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J8" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -3130,9 +3326,9 @@
           <t>Re-evaluate plans following drill and identify additional needs.</t>
         </is>
       </c>
-      <c r="J9" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J9" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3395,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K11" s="51" t="inlineStr"/>
+      <c r="K11" s="51" t="inlineStr">
+        <is>
+          <t>Station facility maintenance monitoring program operational by Q4, with all items inventoried by responsible party, service schedules documented, and internal tracking system active.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="H12" s="41" t="inlineStr">
@@ -3299,7 +3499,7 @@
       </c>
       <c r="G17" s="40" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Terry McCloud</t>
         </is>
       </c>
       <c r="H17" s="41" t="inlineStr">
@@ -3317,7 +3517,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K17" s="42" t="inlineStr"/>
+      <c r="K17" s="42" t="inlineStr">
+        <is>
+          <t>Minimum three additional Hazardous Materials Technician-certified personnel achieved, target hazard pre-plan library complete for all identified city sites, and at least one HOT training or tabletop exercise conducted by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="H18" s="41" t="inlineStr">
@@ -3433,7 +3637,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K22" s="51" t="inlineStr"/>
+      <c r="K22" s="51" t="inlineStr">
+        <is>
+          <t>PPE inventory assessed, minimum reserve standards established, lifecycle replacement model documented with annual funding projections, and sustainable PPE readiness program implemented by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="H23" s="41" t="inlineStr">
@@ -3549,7 +3757,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K27" s="58" t="inlineStr"/>
+      <c r="K27" s="58" t="inlineStr">
+        <is>
+          <t>Needs assessment complete, logistics resource hub program developed with inventory management system installed, SOGs documented, personnel trained, and initial effectiveness evaluation completed by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="H28" s="41" t="inlineStr">
@@ -3686,7 +3898,7 @@
       </c>
       <c r="K34" s="42" t="inlineStr">
         <is>
-          <t>Continuity plan adopted with guides for all critical functions. Depends on completion of both PPE program (P1.27.G2) and logistics hubs program (P1.27.G3).</t>
+          <t>Logistics Division continuity plan adopted with position-specific guides and SOPs for all critical functions, cross-training program established, and program appraisal completed by Q4.</t>
         </is>
       </c>
     </row>
@@ -3804,7 +4016,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K39" s="51" t="inlineStr"/>
+      <c r="K39" s="51" t="inlineStr">
+        <is>
+          <t>Structured assessment of all mutual aid agreements, radio interoperability, and CAD integration complete, with prioritized gap report delivered to command staff by Q2.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="H40" s="41" t="inlineStr">
@@ -3903,7 +4119,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K43" s="58" t="inlineStr"/>
+      <c r="K43" s="58" t="inlineStr">
+        <is>
+          <t>Updated mutual aid agreements, joint training protocols, and communications interoperability solutions developed and delivered to all partner agencies for review by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="H44" s="41" t="inlineStr">
@@ -4021,7 +4241,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K49" s="42" t="inlineStr"/>
+      <c r="K49" s="42" t="inlineStr">
+        <is>
+          <t>Fleet readiness and maintenance assessment complete by Q4, with annual maintenance costs calculated per apparatus, downtime measured against manufacturer PM schedules, highest-burden units identified, and KPIs for apparatus availability established.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="H50" s="41" t="inlineStr">
@@ -4137,7 +4361,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K54" s="51" t="inlineStr"/>
+      <c r="K54" s="51" t="inlineStr">
+        <is>
+          <t>Signed updates to all mutual aid agreements executed, minimum one joint interagency training exercise delivered, and communications interoperability verified with all primary mutual aid partners by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="H55" s="41" t="inlineStr">
@@ -4439,7 +4667,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="K6" s="42" t="inlineStr"/>
+      <c r="K6" s="42" t="inlineStr">
+        <is>
+          <t>Written department-wide succession plan adopted by Q4, identifying all personnel eligible to separate within five years, mapping critical position vacancies, and assigning developmental actions to identified successors.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="H7" s="41" t="inlineStr">
@@ -4538,7 +4770,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="K10" s="51" t="inlineStr"/>
+      <c r="K10" s="51" t="inlineStr">
+        <is>
+          <t>Revised Officer Development Program relaunched by Q4 with updated curriculum, current competency expectations aligned to CFAI credentialing categories, and a documented delivery schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="H11" s="41" t="inlineStr">
@@ -4551,9 +4787,9 @@
           <t>Develop education program.</t>
         </is>
       </c>
-      <c r="J11" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J11" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -4568,9 +4804,9 @@
           <t>Collect and review feedback forms.</t>
         </is>
       </c>
-      <c r="J12" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J12" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -4602,9 +4838,9 @@
           <t>FY26</t>
         </is>
       </c>
-      <c r="D14" s="45" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="D14" s="59" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E14" s="54" t="inlineStr">
@@ -4632,12 +4868,16 @@
           <t>Assess current staffing and workload distribution.</t>
         </is>
       </c>
-      <c r="J14" s="50" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K14" s="58" t="inlineStr"/>
+      <c r="J14" s="60" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K14" s="58" t="inlineStr">
+        <is>
+          <t>Documented roles, responsibilities, and reporting structure established for all training division positions, and continuous evaluation framework for workload and span of control implemented by Q3.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="H15" s="41" t="inlineStr">
@@ -4650,9 +4890,9 @@
           <t>Develop clear job descriptions and roles for specific training functions.</t>
         </is>
       </c>
-      <c r="J15" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J15" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -4736,7 +4976,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="K18" s="51" t="inlineStr"/>
+      <c r="K18" s="51" t="inlineStr">
+        <is>
+          <t>Recruitment program operational by Q4 with formal partnerships at a minimum of four local technical schools, functioning online portal, standardized interview questions, documented scoring system, and active recruitment committee.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="H19" s="41" t="inlineStr">
@@ -4871,7 +5115,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K25" s="42" t="inlineStr"/>
+      <c r="K25" s="42" t="inlineStr">
+        <is>
+          <t>Comprehensive EMS organizational evaluation complete by Q3, with findings and specific staffing recommendations for QA/QI, accreditation, and specialty program positions presented to command staff.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="H26" s="41" t="inlineStr">
@@ -4970,7 +5218,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K29" s="51" t="inlineStr"/>
+      <c r="K29" s="51" t="inlineStr">
+        <is>
+          <t>Feasibility report on NPFR-hosted training academy presented to command staff by Q4, with recommended implementation pathway, cost estimates, and regional partnership options documented.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="H30" s="41" t="inlineStr">
@@ -5086,7 +5338,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K34" s="58" t="inlineStr"/>
+      <c r="K34" s="58" t="inlineStr">
+        <is>
+          <t>Sleep health evaluation complete by Q4, with findings on crew-quarters configuration, personnel survey results, and facility and policy recommendations presented to command staff.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="H35" s="41" t="inlineStr">
@@ -5202,7 +5458,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K39" s="51" t="inlineStr"/>
+      <c r="K39" s="51" t="inlineStr">
+        <is>
+          <t>Internal communication program fully operational by Q4, with all stations visited a minimum of twice, quarterly department periodical published, and digital communication platform active for shift-based staff.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="H40" s="41" t="inlineStr">
@@ -5337,7 +5597,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K46" s="42" t="inlineStr"/>
+      <c r="K46" s="42" t="inlineStr">
+        <is>
+          <t>EMS supervisory evaluation complete by Q4, with findings on field coverage effectiveness, clinical oversight opportunities, and implementation recommendations for future supervisory positions presented to command staff.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="H47" s="41" t="inlineStr">
@@ -5425,7 +5689,7 @@
       </c>
       <c r="E51" s="44" t="inlineStr">
         <is>
-          <t>P2.27.G3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F51" s="46" t="inlineStr">
@@ -5453,7 +5717,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K51" s="51" t="inlineStr"/>
+      <c r="K51" s="51" t="inlineStr">
+        <is>
+          <t>Formal partnership agreements executed with a minimum of four regional educational institutions by Q4, shared-resource access protocols documented, and joint recruitment pipeline established with at least two institutions.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="H52" s="41" t="inlineStr">
@@ -5552,7 +5820,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K55" s="58" t="inlineStr"/>
+      <c r="K55" s="58" t="inlineStr">
+        <is>
+          <t>NPFR Training Academy established by Q4, with facility and partnership agreements in place and a minimum of one formally structured training program delivered to internal personnel with outcomes documented.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="H56" s="41" t="inlineStr">
@@ -5668,7 +5940,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K60" s="51" t="inlineStr"/>
+      <c r="K60" s="51" t="inlineStr">
+        <is>
+          <t>Individual sleeping room retrofit at Brix station complete by Q4, station-level sleep hygiene protocols adopted, and personnel survey conducted to assess improvement in self-reported sleep quality.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="H61" s="41" t="inlineStr">
@@ -5803,7 +6079,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K67" s="42" t="inlineStr"/>
+      <c r="K67" s="42" t="inlineStr">
+        <is>
+          <t>90% or greater professional credentialing of all applicable positions documented by Q4, with individual completion plans on file for all remaining uncredentialed personnel.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="H68" s="41" t="inlineStr">
@@ -5902,7 +6182,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K71" s="51" t="inlineStr"/>
+      <c r="K71" s="51" t="inlineStr">
+        <is>
+          <t>Workforce growth plan presented to command staff by Q4, projecting staffing needs through FY32 with a phased onboarding model covering hiring timeline, employment terms, career progression, and retention strategies.</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="H72" s="41" t="inlineStr">
@@ -6001,7 +6285,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K75" s="58" t="inlineStr"/>
+      <c r="K75" s="58" t="inlineStr">
+        <is>
+          <t>Financial plan addressing projected staffing growth through FY32 presented for command staff adoption by Q4, with position cost modeling, identified funding sources, and phased hiring timeline aligned to call volume thresholds.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="H76" s="41" t="inlineStr">
@@ -6083,7 +6371,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K78" s="51" t="inlineStr"/>
+      <c r="K78" s="51" t="inlineStr">
+        <is>
+          <t>Recognized training center status achieved, minimum two training sessions hosted, collaborative training events with external agencies increased 50% over FY28 baseline, and external trainee participation in NPFR-led courses increased 30% by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="H79" s="41" t="inlineStr">
@@ -6409,9 +6701,9 @@
           <t>FY26</t>
         </is>
       </c>
-      <c r="D6" s="53" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -6439,12 +6731,16 @@
           <t>Access and compile data from ImageTrend, police reporting, GIS, Mobile-Eyes, and regional sources.</t>
         </is>
       </c>
-      <c r="J6" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K6" s="42" t="inlineStr"/>
+      <c r="J6" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K6" s="42" t="inlineStr">
+        <is>
+          <t>Ranked baseline risk report identifying highest-priority program areas delivered to the CRR team by Q2, drawing from a minimum of five data sources.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="H7" s="41" t="inlineStr">
@@ -6457,9 +6753,9 @@
           <t>Organize data and rank by importance, financial impact, and organizational capacity.</t>
         </is>
       </c>
-      <c r="J7" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J7" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -6508,9 +6804,9 @@
           <t>FY26</t>
         </is>
       </c>
-      <c r="D10" s="45" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E10" s="44" t="inlineStr">
@@ -6538,12 +6834,16 @@
           <t>Establish programs based on greatest identified need from data evaluation.</t>
         </is>
       </c>
-      <c r="J10" s="50" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K10" s="51" t="inlineStr"/>
+      <c r="J10" s="60" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K10" s="51" t="inlineStr">
+        <is>
+          <t>Elementary School CRR Education program and Senior Public Education program both operational by Q4, with baseline data collection underway for each.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="H11" s="41" t="inlineStr">
@@ -6556,9 +6856,9 @@
           <t>Formalize Elementary School CRR Education program.</t>
         </is>
       </c>
-      <c r="J11" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J11" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -6573,9 +6873,9 @@
           <t>Formalize Senior Public Education program.</t>
         </is>
       </c>
-      <c r="J12" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J12" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6961,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K16" s="42" t="inlineStr"/>
+      <c r="K16" s="42" t="inlineStr">
+        <is>
+          <t>Targeted EMS prevention initiatives addressing CPR, falls, stroke awareness, drowning prevention, and severe weather preparedness launched by Q3, with performance measures established for all EMS-related CRR activities.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="H17" s="41" t="inlineStr">
@@ -6777,7 +7081,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K21" s="51" t="inlineStr"/>
+      <c r="K21" s="51" t="inlineStr">
+        <is>
+          <t>Minimum three new CRR program policies with supporting content complete by Q1, Programs 1 and 2 operational by Q3, and Programs 3 and 4 operational by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="H22" s="41" t="inlineStr">
@@ -6876,7 +7184,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K25" s="58" t="inlineStr"/>
+      <c r="K25" s="58" t="inlineStr">
+        <is>
+          <t>CRR staffing capacity analysis presented to command staff by Q3, and interim capacity solutions including cross-training and volunteer engagement established by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="H26" s="41" t="inlineStr">
@@ -7011,7 +7323,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K32" s="42" t="inlineStr"/>
+      <c r="K32" s="42" t="inlineStr">
+        <is>
+          <t>Written report documenting CRR and EMS program strengths, weaknesses, and data-driven improvement recommendations delivered by Q4, based on updated multi-source data analysis.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="H33" s="41" t="inlineStr">
@@ -7110,7 +7426,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K36" s="51" t="inlineStr"/>
+      <c r="K36" s="51" t="inlineStr">
+        <is>
+          <t>Fire Explorer and Cadet pathway program established in partnership with a minimum of two local high schools by Q4, annual station visits and career days implemented, and formal program appraisal of Cadet Program completed.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="H37" s="41" t="inlineStr">
@@ -7226,7 +7546,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K41" s="58" t="inlineStr"/>
+      <c r="K41" s="58" t="inlineStr">
+        <is>
+          <t>Community Outreach Team established with defined structure and trained membership by Q4, and a minimum of two community events delivered.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="H42" s="41" t="inlineStr">
@@ -7344,7 +7668,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K47" s="42" t="inlineStr"/>
+      <c r="K47" s="42" t="inlineStr">
+        <is>
+          <t>Expansion of the three highest-performing CRR programs documented and reported by Q2, with measurable increases in reach, delivery frequency, or target population coverage.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="H48" s="41" t="inlineStr">
@@ -7409,7 +7737,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K49" s="51" t="inlineStr"/>
+      <c r="K49" s="51" t="inlineStr">
+        <is>
+          <t>Improvement plans for the three lowest-performing CRR programs implemented and outcomes assessed by Q3.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="H50" s="41" t="inlineStr">
@@ -7491,7 +7823,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K52" s="58" t="inlineStr"/>
+      <c r="K52" s="58" t="inlineStr">
+        <is>
+          <t>Adapted or new program delivery operational in a minimum of two identified underserved geographic areas or demographic gap populations by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="H53" s="41" t="inlineStr">
@@ -7765,9 +8101,9 @@
           <t>FY26</t>
         </is>
       </c>
-      <c r="D6" s="53" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -7792,7 +8128,7 @@
       </c>
       <c r="I6" s="25" t="inlineStr">
         <is>
-          <t>Formalize Accreditation SOG.</t>
+          <t>Strategic Plan adopted by the AHJ</t>
         </is>
       </c>
       <c r="J6" s="32" t="inlineStr">
@@ -7800,7 +8136,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K6" s="42" t="inlineStr"/>
+      <c r="K6" s="42" t="inlineStr">
+        <is>
+          <t>CFAI candidate application submitted by Q4, with Accreditation SOG formalized and documented proof of compliance gathered across all applicable categories.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="H7" s="41" t="inlineStr">
@@ -7813,9 +8153,9 @@
           <t>Implement processes and move toward best practice alignment.</t>
         </is>
       </c>
-      <c r="J7" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J7" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -7830,9 +8170,9 @@
           <t>Gather proof of compliance.</t>
         </is>
       </c>
-      <c r="J8" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J8" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -7847,9 +8187,9 @@
           <t>Achieve CFAI applicant status.</t>
         </is>
       </c>
-      <c r="J9" s="32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="J9" s="34" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -7861,7 +8201,7 @@
       </c>
       <c r="I10" s="25" t="inlineStr">
         <is>
-          <t>Deliver training on SOG including outlier response time policies.</t>
+          <t>CRA SOC Adopted by the AHJ</t>
         </is>
       </c>
       <c r="J10" s="32" t="inlineStr">
@@ -7873,7 +8213,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="43" t="inlineStr">
         <is>
-          <t>P4.26.G2 ★</t>
+          <t>P4.26.G2</t>
         </is>
       </c>
       <c r="C11" s="44" t="inlineStr">
@@ -7916,7 +8256,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="K11" s="51" t="inlineStr"/>
+      <c r="K11" s="51" t="inlineStr">
+        <is>
+          <t>ISO 1 annual compliance package complete by Q4, with all required data documented and site visit readiness package delivered.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="H12" s="41" t="inlineStr">
@@ -8032,7 +8376,11 @@
           <t>Complete</t>
         </is>
       </c>
-      <c r="K16" s="58" t="inlineStr"/>
+      <c r="K16" s="58" t="inlineStr">
+        <is>
+          <t>Mission Lifeline Gold Rating application submitted by Q4 with supporting quarterly cardiac care data and protocol alignment verified.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="H17" s="41" t="inlineStr">
@@ -8150,7 +8498,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K22" s="42" t="inlineStr"/>
+      <c r="K22" s="42" t="inlineStr">
+        <is>
+          <t>All assigned accreditation tasks completed, 11th edition manual requirements incorporated, and next defined CFAI accreditation milestone reached by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="H23" s="41" t="inlineStr">
@@ -8206,7 +8558,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="43" t="inlineStr">
         <is>
-          <t>P4.27.G2 ★</t>
+          <t>P4.27.G2</t>
         </is>
       </c>
       <c r="C26" s="44" t="inlineStr">
@@ -8221,12 +8573,12 @@
       </c>
       <c r="E26" s="44" t="inlineStr">
         <is>
-          <t>P4.26.G2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="46" t="inlineStr">
         <is>
-          <t>Complete CAAS re-accreditation by incorporating all 4th edition manual requirements, obtaining annual proofs of compliance across all applicable categories, submitting the re-accreditation application, completing the PedReady renewal, and achieving a successful on-site review by Q4.</t>
+          <t>Complete CAAS re-accreditation by incorporating all 4th edition manual requirements, obtaining annual proofs of compliance across all applicable categories, submitting the re-accreditation application, and achieving a successful on-site review by Q4.</t>
         </is>
       </c>
       <c r="G26" s="47" t="inlineStr">
@@ -8249,7 +8601,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K26" s="51" t="inlineStr"/>
+      <c r="K26" s="51" t="inlineStr">
+        <is>
+          <t>CAAS re-accreditation achieved by Q4, with 4th edition manual requirements incorporated, all annual proofs of compliance gathered, re-accreditation application submitted, and successful on-site review conducted.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="H27" s="41" t="inlineStr">
@@ -8365,7 +8721,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K31" s="58" t="inlineStr"/>
+      <c r="K31" s="58" t="inlineStr">
+        <is>
+          <t>ALS coverage improvement plan with specific resource and staffing recommendations presented to executive leadership by Q4, based on completed response time analysis, coverage gap mapping, and staffing model evaluation.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="H32" s="41" t="inlineStr">
@@ -8455,7 +8815,7 @@
       </c>
       <c r="E37" s="15" t="inlineStr">
         <is>
-          <t>P4.27.G2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F37" s="39" t="inlineStr">
@@ -8483,7 +8843,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K37" s="42" t="inlineStr"/>
+      <c r="K37" s="42" t="inlineStr">
+        <is>
+          <t>Centralized digital records management system operational by Q4, with complete record inventory documented, all active records migrated, and records meeting retention requirements dispositioned with the Clerk's office.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="H38" s="41" t="inlineStr">
@@ -8582,7 +8946,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K41" s="51" t="inlineStr"/>
+      <c r="K41" s="51" t="inlineStr">
+        <is>
+          <t>MIH implementation recommendation presented to command staff by Q4, with completed operational framework, target population analysis, partner identification, performance measures, referral pathways, and financial and staffing feasibility evaluation.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="H42" s="41" t="inlineStr">
@@ -8698,7 +9066,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K46" s="58" t="inlineStr"/>
+      <c r="K46" s="58" t="inlineStr">
+        <is>
+          <t>Prioritized implementation strategy with go/no-go recommendations for a minimum of two advanced EMS service models presented to executive leadership by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="H47" s="41" t="inlineStr">
@@ -8833,7 +9205,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K53" s="42" t="inlineStr"/>
+      <c r="K53" s="42" t="inlineStr">
+        <is>
+          <t>Historical and Archive Committee established with formal mandate, recruited membership, and initial inventory of historical items complete by Q2; agency performance standards implemented with documented compliance tracking process by Q4.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="H54" s="41" t="inlineStr">
@@ -8966,7 +9342,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K59" s="51" t="inlineStr"/>
+      <c r="K59" s="51" t="inlineStr">
+        <is>
+          <t>MIH pilot program launched by Q4 serving identified high-utilizer or at-risk populations, with formal healthcare partnerships established, policy and documentation frameworks complete, and quarterly outcomes tracking initiated.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="H60" s="41" t="inlineStr">
@@ -9065,7 +9445,11 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K63" s="58" t="inlineStr"/>
+      <c r="K63" s="58" t="inlineStr">
+        <is>
+          <t>Minimum one advanced EMS service model implemented by Q4, with documented operational framework, trained personnel, structured outcomes tracking, and first-year performance report delivered to command staff.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="H64" s="41" t="inlineStr">
@@ -9233,7 +9617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9409,34 +9793,34 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>P2.28.G2</t>
+          <t>P2.28.G4</t>
         </is>
       </c>
       <c r="E10" s="25" t="inlineStr">
         <is>
-          <t>Execute formal partnership agreements with a minimum of four regional educational institutions, establish documented shared-resource access protocols for training infrastructure, and develop a joint recruitment pipeline pathway with at least two institutions by Q4.</t>
+          <t>Implement the sleep health improvement recommendations identified in the FY27 sleep study, including retrofit of individual sleeping rooms at Brix station and adoption of station-level sleep hygiene protocols, with all primary facility modifications complete by Q4.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>P2.27.G3 ★</t>
+          <t>P2.28.G1 ★</t>
         </is>
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Complete a formal evaluation of sleep health challenges facing shift-based personnel, including review of current crew-quarters configuration, existing research on firefighter sleep deprivation, and peer agency solutions, and present findings with recommendations to command staff by Q4.</t>
+          <t>Complete a formal evaluation of EMS supervisory roles, field coverage effectiveness, and future deployment models, and present findings with implementation recommendations to command staff by Q4.</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>P2.28.G4</t>
+          <t>P2.29.G2</t>
         </is>
       </c>
       <c r="E11" s="30" t="inlineStr">
         <is>
-          <t>Implement the sleep health improvement recommendations identified in the FY27 sleep study, including retrofit of individual sleeping rooms at Brix station and adoption of station-level sleep hygiene protocols, with all primary facility modifications complete by Q4.</t>
+          <t>Develop and present a workforce growth plan that identifies staffing needs through FY32 based on call volume trends and community growth data, includes a phased onboarding model with hiring timeline, employment terms, career progression, and retention strategies, by Q4.</t>
         </is>
       </c>
     </row>
@@ -9453,56 +9837,56 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>P2.29.G2</t>
+          <t>P2.29.G3</t>
         </is>
       </c>
       <c r="E12" s="25" t="inlineStr">
         <is>
-          <t>Develop and present a workforce growth plan that identifies staffing needs through FY32 based on call volume trends and community growth data, includes a phased onboarding model with hiring timeline, employment terms, career progression, and retention strategies, by Q4.</t>
+          <t>Develop a financial plan addressing projected staffing growth needs through FY32, incorporating position cost modeling, identified funding sources, and a phased hiring timeline aligned to call volume thresholds, and present for command staff adoption by Q4.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>P2.28.G1 ★</t>
+          <t>P2.28.G3 ★</t>
         </is>
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>Complete a formal evaluation of EMS supervisory roles, field coverage effectiveness, and future deployment models, and present findings with implementation recommendations to command staff by Q4.</t>
+          <t>Establish a functioning NPFR Training Academy by implementing the pathway recommended in the FY27 evaluation, securing necessary facility arrangements and partnerships, and delivering a minimum of one formally structured training program to internal personnel by Q4.</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>P2.29.G3</t>
+          <t>P2.29.G4</t>
         </is>
       </c>
       <c r="E13" s="30" t="inlineStr">
         <is>
-          <t>Develop a financial plan addressing projected staffing growth needs through FY32, incorporating position cost modeling, identified funding sources, and a phased hiring timeline aligned to call volume thresholds, and present for command staff adoption by Q4.</t>
+          <t>Achieve recognized training center status, host a minimum of two training sessions, increase collaborative training events with external agencies by 50% over the FY28 baseline, and increase external trainee participation in NPFR-led courses by 30% by Q4.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>P2.28.G3 ★</t>
+          <t>P3.26.G1 ★</t>
         </is>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>Establish a functioning NPFR Training Academy by implementing the pathway recommended in the FY27 evaluation, securing necessary facility arrangements and partnerships, and delivering a minimum of one formally structured training program to internal personnel by Q4.</t>
+          <t>Gather, organize, and evaluate community risk data from five sources including ImageTrend, police reporting, GIS, Mobile-Eyes, and regional data, and deliver a ranked baseline risk report identifying highest-priority program areas to the CRR team by Q2.</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>P2.29.G4</t>
+          <t>P3.26.G2</t>
         </is>
       </c>
       <c r="E14" s="25" t="inlineStr">
         <is>
-          <t>Achieve recognized training center status, host a minimum of two training sessions, increase collaborative training events with external agencies by 50% over the FY28 baseline, and increase external trainee participation in NPFR-led courses by 30% by Q4.</t>
+          <t>Design and launch two new community risk reduction programs targeting the highest-priority risk categories identified in the FY26 baseline report, including a formalized Elementary School CRR Education program and a Senior Public Education program, with both programs operational and baseline data collection underway by Q4.</t>
         </is>
       </c>
     </row>
@@ -9519,78 +9903,78 @@
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>P3.26.G2</t>
+          <t>P3.27.G2</t>
         </is>
       </c>
       <c r="E15" s="30" t="inlineStr">
         <is>
-          <t>Design and launch two new community risk reduction programs targeting the highest-priority risk categories identified in the FY26 baseline report, including a formalized Elementary School CRR Education program and a Senior Public Education program, with both programs operational and baseline data collection underway by Q4.</t>
+          <t>Develop a minimum of three new CRR program policies with supporting content by Q1, and complete phased rollout of a minimum of four CRR programs with Programs 1 and 2 operational by Q3 and Programs 3 and 4 operational by Q4.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>P3.26.G1 ★</t>
+          <t>P3.27.G2 ★</t>
         </is>
       </c>
       <c r="C16" s="25" t="inlineStr">
         <is>
-          <t>Gather, organize, and evaluate community risk data from five sources including ImageTrend, police reporting, GIS, Mobile-Eyes, and regional data, and deliver a ranked baseline risk report identifying highest-priority program areas to the CRR team by Q2.</t>
+          <t>Develop a minimum of three new CRR program policies with supporting content by Q1, and complete phased rollout of a minimum of four CRR programs with Programs 1 and 2 operational by Q3 and Programs 3 and 4 operational by Q4.</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>P3.27.G2</t>
+          <t>P3.28.G1</t>
         </is>
       </c>
       <c r="E16" s="25" t="inlineStr">
         <is>
-          <t>Develop a minimum of three new CRR program policies with supporting content by Q1, and complete phased rollout of a minimum of four CRR programs with Programs 1 and 2 operational by Q3 and Programs 3 and 4 operational by Q4.</t>
+          <t>Gather updated CRR and EMS program data from all relevant sources, analyze incident trends to identify high-risk populations and areas, and deliver a written report documenting program strengths, weaknesses, and data-driven recommendations for program improvement by Q4.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>P3.27.G2 ★</t>
+          <t>P3.27.G3 ★</t>
         </is>
       </c>
       <c r="C17" s="30" t="inlineStr">
         <is>
-          <t>Develop a minimum of three new CRR program policies with supporting content by Q1, and complete phased rollout of a minimum of four CRR programs with Programs 1 and 2 operational by Q3 and Programs 3 and 4 operational by Q4.</t>
+          <t>Complete a CRR staffing capacity analysis relative to identified program delivery requirements, present a staffing needs recommendation to command staff by Q3, and establish interim capacity solutions including cross-training and volunteer engagement by Q4.</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>P3.28.G1</t>
+          <t>P3.28.G3</t>
         </is>
       </c>
       <c r="E17" s="30" t="inlineStr">
         <is>
-          <t>Gather updated CRR and EMS program data from all relevant sources, analyze incident trends to identify high-risk populations and areas, and deliver a written report documenting program strengths, weaknesses, and data-driven recommendations for program improvement by Q4.</t>
+          <t>Establish a Community Outreach Team of trained firefighters capable of supporting public education presentations and community events, with a defined team structure, trained membership, and a minimum of two community events delivered by Q4.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>P3.27.G3 ★</t>
+          <t>P3.28.G1 ★</t>
         </is>
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t>Complete a CRR staffing capacity analysis relative to identified program delivery requirements, present a staffing needs recommendation to command staff by Q3, and establish interim capacity solutions including cross-training and volunteer engagement by Q4.</t>
+          <t>Gather updated CRR and EMS program data from all relevant sources, analyze incident trends to identify high-risk populations and areas, and deliver a written report documenting program strengths, weaknesses, and data-driven recommendations for program improvement by Q4.</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>P3.28.G3</t>
+          <t>P3.29.G1</t>
         </is>
       </c>
       <c r="E18" s="25" t="inlineStr">
         <is>
-          <t>Establish a Community Outreach Team of trained firefighters capable of supporting public education presentations and community events, with a defined team structure, trained membership, and a minimum of two community events delivered by Q4.</t>
+          <t>Expand the three highest-performing CRR programs identified through FY28 data analysis by increasing reach, delivery frequency, or target population coverage, with documented expansion outcomes reported by Q2.</t>
         </is>
       </c>
     </row>
@@ -9607,164 +9991,98 @@
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>P3.29.G1</t>
+          <t>P3.29.G2</t>
         </is>
       </c>
       <c r="E19" s="30" t="inlineStr">
         <is>
-          <t>Expand the three highest-performing CRR programs identified through FY28 data analysis by increasing reach, delivery frequency, or target population coverage, with documented expansion outcomes reported by Q2.</t>
+          <t>Implement targeted improvement plans for the three lowest-performing CRR programs identified through FY28 data analysis, with all improvement actions executed and outcomes assessed by Q3.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>P3.28.G1 ★</t>
+          <t>P4.26.G1 ★</t>
         </is>
       </c>
       <c r="C20" s="25" t="inlineStr">
         <is>
-          <t>Gather updated CRR and EMS program data from all relevant sources, analyze incident trends to identify high-risk populations and areas, and deliver a written report documenting program strengths, weaknesses, and data-driven recommendations for program improvement by Q4.</t>
+          <t>Achieve CFAI accreditation candidate status by formalizing the Accreditation SOG, implementing compliant processes across all applicable categories, gathering documented proof of compliance, and submitting the CFAI candidate application by Q4.</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>P3.29.G2</t>
+          <t>P4.27.G1</t>
         </is>
       </c>
       <c r="E20" s="25" t="inlineStr">
         <is>
-          <t>Implement targeted improvement plans for the three lowest-performing CRR programs identified through FY28 data analysis, with all improvement actions executed and outcomes assessed by Q3.</t>
+          <t>Advance CFAI accreditation progress by completing all assigned tasks, incorporating 11th edition manual requirements, gathering ongoing proof of compliance across all categories, and reaching the next defined accreditation milestone by Q4.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>P4.26.G1 ★</t>
+          <t>P4.27.G1 ★</t>
         </is>
       </c>
       <c r="C21" s="30" t="inlineStr">
         <is>
-          <t>Achieve CFAI accreditation candidate status by formalizing the Accreditation SOG, implementing compliant processes across all applicable categories, gathering documented proof of compliance, and submitting the CFAI candidate application by Q4.</t>
+          <t>Advance CFAI accreditation progress by completing all assigned tasks, incorporating 11th edition manual requirements, gathering ongoing proof of compliance across all categories, and reaching the next defined accreditation milestone by Q4.</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>P4.27.G1</t>
+          <t>P4.29.G1</t>
         </is>
       </c>
       <c r="E21" s="30" t="inlineStr">
         <is>
-          <t>Advance CFAI accreditation progress by completing all assigned tasks, incorporating 11th edition manual requirements, gathering ongoing proof of compliance across all categories, and reaching the next defined accreditation milestone by Q4.</t>
+          <t>Establish a Historical and Archive Committee with a formal mandate, recruited membership, and completed initial inventory of historical items by Q2, and implement agency performance standards with a documented compliance tracking and evaluation process by Q4.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>P4.26.G2 ★</t>
+          <t>P4.28.G2 ★</t>
         </is>
       </c>
       <c r="C22" s="25" t="inlineStr">
         <is>
-          <t>Complete all ISO 1 annual compliance requirements including needs assessment, departmental collaboration, data documentation, and proof of compliance, and deliver a site visit readiness package by Q4.</t>
+          <t>Develop a Mobile Integrated Healthcare operational framework including target population analysis, partner identification, performance measures, referral pathways, and a financial and staffing feasibility evaluation, and present an MIH implementation recommendation to command staff by Q4.</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>P4.27.G2</t>
+          <t>P4.29.G2</t>
         </is>
       </c>
       <c r="E22" s="25" t="inlineStr">
         <is>
-          <t>Complete CAAS re-accreditation by incorporating all 4th edition manual requirements, obtaining annual proofs of compliance across all applicable categories, submitting the re-accreditation application, completing the PedReady renewal, and achieving a successful on-site review by Q4.</t>
+          <t>Implement the Mobile Integrated Healthcare program by establishing formal healthcare partnerships, completing all policy and documentation frameworks, launching a pilot serving identified high-utilizer or at-risk populations by Q4, and initiating quarterly outcomes tracking.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>P4.27.G2 ★</t>
+          <t>P4.28.G3 ★</t>
         </is>
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>Complete CAAS re-accreditation by incorporating all 4th edition manual requirements, obtaining annual proofs of compliance across all applicable categories, submitting the re-accreditation application, completing the PedReady renewal, and achieving a successful on-site review by Q4.</t>
+          <t>Evaluate the demand, financial viability, staffing requirements, and operational feasibility of a minimum of two advanced EMS service models, and present a prioritized implementation strategy with go/no-go recommendations to executive leadership by Q4.</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>P4.28.G1</t>
+          <t>P4.29.G3</t>
         </is>
       </c>
       <c r="E23" s="30" t="inlineStr">
-        <is>
-          <t>Develop a centralized digital records management system including a complete record inventory, file mapping, access controls, migration of all active records not meeting retention, and completed disposition of records that have met retention requirements with the Clerk's office by Q4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>P4.27.G1 ★</t>
-        </is>
-      </c>
-      <c r="C24" s="25" t="inlineStr">
-        <is>
-          <t>Advance CFAI accreditation progress by completing all assigned tasks, incorporating 11th edition manual requirements, gathering ongoing proof of compliance across all categories, and reaching the next defined accreditation milestone by Q4.</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>P4.29.G1</t>
-        </is>
-      </c>
-      <c r="E24" s="25" t="inlineStr">
-        <is>
-          <t>Establish a Historical and Archive Committee with a formal mandate, recruited membership, and completed initial inventory of historical items by Q2, and implement agency performance standards with a documented compliance tracking and evaluation process by Q4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>P4.28.G2 ★</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t>Develop a Mobile Integrated Healthcare operational framework including target population analysis, partner identification, performance measures, referral pathways, and a financial and staffing feasibility evaluation, and present an MIH implementation recommendation to command staff by Q4.</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>P4.29.G2</t>
-        </is>
-      </c>
-      <c r="E25" s="30" t="inlineStr">
-        <is>
-          <t>Implement the Mobile Integrated Healthcare program by establishing formal healthcare partnerships, completing all policy and documentation frameworks, launching a pilot serving identified high-utilizer or at-risk populations by Q4, and initiating quarterly outcomes tracking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>P4.28.G3 ★</t>
-        </is>
-      </c>
-      <c r="C26" s="25" t="inlineStr">
-        <is>
-          <t>Evaluate the demand, financial viability, staffing requirements, and operational feasibility of a minimum of two advanced EMS service models, and present a prioritized implementation strategy with go/no-go recommendations to executive leadership by Q4.</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>P4.29.G3</t>
-        </is>
-      </c>
-      <c r="E26" s="25" t="inlineStr">
         <is>
           <t>Implement a minimum of one advanced EMS service model based on FY28 feasibility findings with a documented operational framework, trained personnel, and structured outcomes tracking, and deliver a first-year performance report to command staff by Q4.</t>
         </is>
@@ -9785,7 +10103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9834,43 +10152,51 @@
     <row r="4" ht="20" customHeight="1">
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>2026-06-12T21:43:01.168Z</t>
+          <t>2026-06-14T11:54:26.362Z</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>edit_pillar</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr"/>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>P4.26.G1</t>
+        </is>
+      </c>
       <c r="E4" s="25" t="inlineStr">
         <is>
-          <t>P4 â†’ P4: Professional Standards and Service Excellence</t>
+          <t>Implement processes and move toward best practice alignment.  not-started → complete</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>2026-06-12T21:42:54.225Z</t>
+          <t>2026-06-14T11:54:25.872Z</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>edit_pillar</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr"/>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>P4.26.G1</t>
+        </is>
+      </c>
       <c r="E5" s="30" t="inlineStr">
         <is>
-          <t>P3 â†’ P3: Community Risk Reduction and Public Education</t>
+          <t>Gather proof of compliance.  not-started → complete</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>2026-06-12T21:33:57.627Z</t>
+          <t>2026-06-14T11:54:24.641Z</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -9880,19 +10206,19 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>P2.26.G1</t>
+          <t>P4.26.G1</t>
         </is>
       </c>
       <c r="E6" s="25" t="inlineStr">
         <is>
-          <t>Identify personnel leaving within the next five years.  not-started → complete</t>
+          <t>Achieve CFAI applicant status.  not-started → complete</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>2026-06-12T21:33:56.329Z</t>
+          <t>2026-06-14T11:54:21.996Z</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -9902,19 +10228,19 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>P2.26.G2</t>
+          <t>P3.26.G2</t>
         </is>
       </c>
       <c r="E7" s="30" t="inlineStr">
         <is>
-          <t>Update and revise job descriptions.  not-started → complete</t>
+          <t>Formalize Senior Public Education program.  not-started → complete</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>2026-06-12T21:33:48.410Z</t>
+          <t>2026-06-14T11:54:21.652Z</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -9924,32 +10250,398 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>P1.26.G1</t>
+          <t>P3.26.G2</t>
         </is>
       </c>
       <c r="E8" s="25" t="inlineStr">
         <is>
-          <t>Develop a response plan for each identified threat.  not-started → complete</t>
+          <t>Formalize Elementary School CRR Education program.  not-started → complete</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="18" t="inlineStr">
         <is>
+          <t>2026-06-14T11:54:20.987Z</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>P3.26.G2</t>
+        </is>
+      </c>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>Establish programs based on greatest identified need from da  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:54:09.487Z</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>P3.26.G1</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>Organize data and rank by importance, financial impact, and   not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:54:09.076Z</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>P3.26.G1</t>
+        </is>
+      </c>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>Access and compile data from ImageTrend, police reporting, G  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:54:05.576Z</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>P2.26.G3</t>
+        </is>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>Develop clear job descriptions and roles for specific traini  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:54:05.057Z</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>P2.26.G3</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>Assess current staffing and workload distribution.  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:54:00.882Z</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>P2.26.G2</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>Relaunch revised ODP with defined enrollment criteria and de  complete → not-started</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:53:56.405Z</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>P2.26.G2</t>
+        </is>
+      </c>
+      <c r="E15" s="30" t="inlineStr">
+        <is>
+          <t>Relaunch revised ODP with defined enrollment criteria and de  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:53:54.938Z</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>P2.26.G2</t>
+        </is>
+      </c>
+      <c r="E16" s="25" t="inlineStr">
+        <is>
+          <t>Collect and review feedback forms.  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:53:52.167Z</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>P2.26.G2</t>
+        </is>
+      </c>
+      <c r="E17" s="30" t="inlineStr">
+        <is>
+          <t>Develop education program.  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:53:05.361Z</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>P1.26.G1</t>
+        </is>
+      </c>
+      <c r="E18" s="25" t="inlineStr">
+        <is>
+          <t>Re-evaluate plans following drill and identify additional ne  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-14T11:53:04.624Z</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>P1.26.G1</t>
+        </is>
+      </c>
+      <c r="E19" s="30" t="inlineStr">
+        <is>
+          <t>Plan and conduct a large-scale drill including active shoote  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-13T17:14:02.045Z</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>edit_goal</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>P1.27.G1</t>
+        </is>
+      </c>
+      <c r="E20" s="25" t="inlineStr">
+        <is>
+          <t>Edited: year=FY27, domain=Incident Preparedness, predecessor=none</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-12T21:43:01.168Z</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>edit_pillar</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>P4 â†’ P4: Professional Standards and Service Excellence</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-12T21:42:54.225Z</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>edit_pillar</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr"/>
+      <c r="E22" s="25" t="inlineStr">
+        <is>
+          <t>P3 â†’ P3: Community Risk Reduction and Public Education</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-12T21:33:57.627Z</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>P2.26.G1</t>
+        </is>
+      </c>
+      <c r="E23" s="30" t="inlineStr">
+        <is>
+          <t>Identify personnel leaving within the next five years.  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-12T21:33:56.329Z</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>P2.26.G2</t>
+        </is>
+      </c>
+      <c r="E24" s="25" t="inlineStr">
+        <is>
+          <t>Update and revise job descriptions.  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-12T21:33:48.410Z</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>P1.26.G1</t>
+        </is>
+      </c>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Develop a response plan for each identified threat.  not-started → complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="15" t="inlineStr">
+        <is>
           <t>2026-06-12T21:33:47.803Z</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>P1.26.G1</t>
         </is>
       </c>
-      <c r="E9" s="30" t="inlineStr">
+      <c r="E26" s="25" t="inlineStr">
         <is>
           <t>Identify major incident threat types across all hazard types  not-started → complete</t>
         </is>

</xml_diff>